<commit_message>
Task 2: Integration Testing - finished
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/lib/controller/__tests__/it/exercise-controller/createExercise-it-form.xlsx
+++ b/Exam/gymtrackerpro/lib/controller/__tests__/it/exercise-controller/createExercise-it-form.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
   <si>
     <t>Statement: createExercise(data: CreateExerciseInput): Promise&lt;ActionResult&lt;Exercise&gt;&gt; - validates input with Zod, delegates to exerciseService.createExercise(), and returns the persisted entity wrapped in ActionResult.</t>
   </si>
@@ -122,6 +122,26 @@
   </si>
   <si>
     <t>No change</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty database.
+const firstInput: CreateExerciseInput = { name: "Squat", description: "Leg compound", muscleGroup: MuscleGroup.LEGS, equipmentNeeded: Equipment.BARBELL }
+const secondInput: CreateExerciseInput = { name: "Leg Press", description: "Quad focused", muscleGroup: MuscleGroup.LEGS, equipmentNeeded: Equipment.MACHINE }</t>
+  </si>
+  <si>
+    <t>createExercise(firstInput) then createExercise(secondInput)</t>
+  </si>
+  <si>
+    <t>Both calls return { success: true, data: Exercise } with distinct ids</t>
+  </si>
+  <si>
+    <t>Two rows in exercises table; ids are distinct</t>
+  </si>
+  <si>
+    <t>Not yet run</t>
   </si>
   <si>
     <t>Testing</t>
@@ -173,7 +193,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -191,8 +211,11 @@
     <font>
       <color rgb="FF375623"/>
     </font>
+    <font>
+      <color rgb="FF9C0006"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -219,6 +242,11 @@
         <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -239,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -257,6 +285,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -803,12 +834,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="80" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="4" max="4" width="63" customWidth="1"/>
     <col min="5" max="5" width="80" customWidth="1"/>
     <col min="6" max="6" width="67" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
@@ -904,6 +935,29 @@
       </c>
       <c r="G4" s="6" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -924,24 +978,24 @@
     <row r="2" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="4" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="A4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -953,40 +1007,40 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="K5" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -994,40 +1048,40 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>